<commit_message>
fully functional frontend for labs (needs work from parser side)
</commit_message>
<xml_diff>
--- a/uploads/labs.xlsx
+++ b/uploads/labs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\7saka\Desktop\ds_dynamic_schedule\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6088A738-E9C3-4FD7-8A85-EDCCEBF1AA3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47439353-65C7-487F-BEF7-EEA5BA22D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7965" yWindow="3225" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
@@ -284,7 +284,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,6 +380,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -458,7 +465,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -481,38 +488,43 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -815,7 +827,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -826,48 +838,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="10"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="10"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="10"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -901,87 +913,87 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="3"/>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="10" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="5" t="s">
-        <v>15</v>
+      <c r="G7" s="4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="23"/>
-      <c r="D8" s="11" t="s">
+      <c r="C8" s="11"/>
+      <c r="D8" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="21" t="s">
-        <v>21</v>
+      <c r="G8" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="22" t="s">
+      <c r="B9" s="11"/>
+      <c r="C9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="6" t="s">
-        <v>23</v>
+      <c r="D9" s="15"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="8" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="15" t="s">
+      <c r="C10" s="11"/>
+      <c r="D10" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="3"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="23"/>
+      <c r="B11" s="11"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="19" t="s">
+      <c r="D11" s="19"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="16" t="s">
         <v>27</v>
       </c>
       <c r="G11" s="3"/>
@@ -990,47 +1002,47 @@
       <c r="A12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="18" t="s">
         <v>29</v>
       </c>
       <c r="E12" s="3"/>
-      <c r="F12" s="20"/>
+      <c r="F12" s="17"/>
       <c r="G12" s="3"/>
     </row>
     <row r="13" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="15" t="s">
+      <c r="B13" s="11"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="20"/>
+      <c r="F13" s="17"/>
       <c r="G13" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="19" t="s">
+      <c r="E14" s="19"/>
+      <c r="F14" s="16" t="s">
         <v>27</v>
       </c>
       <c r="G14" s="3"/>
@@ -1039,11 +1051,11 @@
       <c r="A15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="20"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="17"/>
       <c r="G15" s="3"/>
     </row>
     <row r="16" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
@@ -1087,19 +1099,19 @@
       <c r="A19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="14" t="s">
         <v>42</v>
       </c>
       <c r="G19" s="3"/>
@@ -1108,27 +1120,27 @@
       <c r="A20" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="12"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="15"/>
       <c r="G20" s="3"/>
     </row>
     <row r="21" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="E21" s="22" t="s">
+      <c r="E21" s="10" t="s">
         <v>33</v>
       </c>
       <c r="F21" s="3"/>
@@ -1138,10 +1150,10 @@
       <c r="A22" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="23"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="11"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
     </row>
@@ -1149,13 +1161,13 @@
       <c r="A23" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="18" t="s">
         <v>25</v>
       </c>
       <c r="E23" s="3"/>
@@ -1166,13 +1178,13 @@
       <c r="A24" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="23"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="15" t="s">
+      <c r="B24" s="11"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="14" t="s">
         <v>44</v>
       </c>
       <c r="G24" s="3"/>
@@ -1181,30 +1193,30 @@
       <c r="A25" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E25" s="16"/>
-      <c r="F25" s="12"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="15"/>
       <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="15" t="s">
+      <c r="B26" s="11"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="14" t="s">
         <v>46</v>
       </c>
       <c r="G26" s="3"/>
@@ -1216,8 +1228,8 @@
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="12"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="15"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1227,8 +1239,8 @@
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="12"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="15"/>
       <c r="G28" s="3"/>
     </row>
     <row r="29" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
@@ -1257,11 +1269,11 @@
       <c r="A31" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="14" t="s">
         <v>49</v>
       </c>
       <c r="C31" s="3"/>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="14" t="s">
         <v>50</v>
       </c>
       <c r="E31" s="3"/>
@@ -1272,13 +1284,13 @@
       <c r="A32" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="12"/>
-      <c r="C32" s="13" t="s">
+      <c r="B32" s="15"/>
+      <c r="C32" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D32" s="12"/>
+      <c r="D32" s="15"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="13" t="s">
+      <c r="F32" s="12" t="s">
         <v>52</v>
       </c>
       <c r="G32" s="3"/>
@@ -1288,14 +1300,14 @@
         <v>24</v>
       </c>
       <c r="B33" s="3"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="11" t="s">
+      <c r="C33" s="13"/>
+      <c r="D33" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="F33" s="14"/>
+      <c r="F33" s="13"/>
       <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1303,11 +1315,11 @@
         <v>26</v>
       </c>
       <c r="B34" s="3"/>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="12"/>
-      <c r="E34" s="23"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="26"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
     </row>
@@ -1316,11 +1328,11 @@
         <v>28</v>
       </c>
       <c r="B35" s="3"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="11" t="s">
+      <c r="C35" s="15"/>
+      <c r="D35" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E35" s="23"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
     </row>
@@ -1330,8 +1342,8 @@
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="22" t="s">
+      <c r="D36" s="15"/>
+      <c r="E36" s="10" t="s">
         <v>57</v>
       </c>
       <c r="F36" s="3"/>
@@ -1341,17 +1353,17 @@
       <c r="A37" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="E37" s="23"/>
-      <c r="F37" s="11" t="s">
+      <c r="E37" s="11"/>
+      <c r="F37" s="14" t="s">
         <v>60</v>
       </c>
       <c r="G37" s="3"/>
@@ -1360,11 +1372,11 @@
       <c r="A38" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="12"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="15"/>
       <c r="E38" s="3"/>
-      <c r="F38" s="12"/>
+      <c r="F38" s="15"/>
       <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -1393,7 +1405,7 @@
       <c r="A41" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="13" t="s">
+      <c r="B41" s="12" t="s">
         <v>53</v>
       </c>
       <c r="C41" s="3"/>
@@ -1406,9 +1418,9 @@
       <c r="A42" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B42" s="14"/>
+      <c r="B42" s="13"/>
       <c r="C42" s="3"/>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="12" t="s">
         <v>62</v>
       </c>
       <c r="E42" s="3"/>
@@ -1419,15 +1431,15 @@
       <c r="A43" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="11" t="s">
+      <c r="B43" s="13"/>
+      <c r="C43" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="D43" s="14"/>
-      <c r="E43" s="11" t="s">
+      <c r="D43" s="13"/>
+      <c r="E43" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="F43" s="11" t="s">
+      <c r="F43" s="14" t="s">
         <v>65</v>
       </c>
       <c r="G43" s="3"/>
@@ -1436,30 +1448,30 @@
       <c r="A44" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="C44" s="12"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
       <c r="G44" s="3"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B45" s="14"/>
-      <c r="C45" s="17" t="s">
+      <c r="B45" s="13"/>
+      <c r="C45" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E45" s="13" t="s">
+      <c r="E45" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="F45" s="13" t="s">
+      <c r="F45" s="12" t="s">
         <v>41</v>
       </c>
       <c r="G45" s="3"/>
@@ -1468,38 +1480,38 @@
       <c r="A46" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
+      <c r="B46" s="13"/>
+      <c r="C46" s="24"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
       <c r="G46" s="3"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B47" s="13" t="s">
+      <c r="B47" s="12" t="s">
         <v>46</v>
       </c>
       <c r="C47" s="3"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="13"/>
+      <c r="F47" s="13"/>
       <c r="G47" s="3"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="14"/>
-      <c r="C48" s="13" t="s">
+      <c r="B48" s="13"/>
+      <c r="C48" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D48" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="E48" s="12" t="s">
         <v>59</v>
       </c>
       <c r="F48" s="3"/>
@@ -1509,11 +1521,11 @@
       <c r="A49" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="13" t="s">
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="12" t="s">
         <v>68</v>
       </c>
       <c r="G49" s="3"/>
@@ -1524,9 +1536,9 @@
       </c>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
       <c r="G50" s="3"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -1542,6 +1554,59 @@
     </row>
   </sheetData>
   <mergeCells count="69">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="F11:F13"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E48:E50"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="E45:E47"/>
+    <mergeCell ref="F45:F47"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F26:F28"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="E13:E15"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="D42:D44"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="E33:E35"/>
     <mergeCell ref="B41:B43"/>
@@ -1558,59 +1623,6 @@
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="D45:D47"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="E13:E15"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="D42:D44"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="E26:E28"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F45:F47"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F26:F28"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="E48:E50"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="E45:E47"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="F11:F13"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="D12:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>